<commit_message>
2026-05-01: scheduler tuning + skill patches
- osi-overnight-runner: yes-with-email cap 3->2, discovery batch 10->5
- osi-prospect-qualification: shallow path engagement gate (12mo reply/meeting required)
- osi-email-sender: TARGET 2->5 with full rationale, leading-blank strip in Step 3B
- Scheduled tasks: weekday cron 7pm/9pm/11pm/1am/3am/5am, weekend every 3hr,
  meeting-followup 9am wkdy, job-change Sun 10pm, NEW email-task-drafts 9am daily,
  morning-skill-sync disabled
- Session logs through 2026-05-01
- Meeting notes through 2026-05-01-amundi
- New: scheduler-cleanup-list.md (70 obsolete tasks for Cowork UI cleanup)
</commit_message>
<xml_diff>
--- a/job-change-tracker.xlsx
+++ b/job-change-tracker.xlsx
@@ -62,7 +62,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +123,12 @@
         <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -210,6 +216,17 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -575,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3003,46 +3020,54 @@
       </c>
     </row>
     <row r="54" ht="40" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>Bob Brizendine</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>Unknown - not loaded</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="inlineStr">
-        <is>
-          <t>Profile not loaded due to lazy-loading on page 1</t>
-        </is>
-      </c>
-      <c r="H54" s="8" t="inlineStr"/>
-      <c r="I54" s="8" t="inlineStr"/>
-      <c r="J54" s="8" t="inlineStr">
-        <is>
-          <t>Page 1, item 25.</t>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>SVP Enterprise Transformation &amp; Deputy Lead Global IT</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>American Honda Motor Company</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>2 tasks created: 4/27 (Touch 1) + 5/11 (Touch 2)</t>
+        </is>
+      </c>
+      <c r="H54" s="25" t="inlineStr">
+        <is>
+          <t>Bob Brizendine - HubSpot</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J54" s="16" t="inlineStr">
+        <is>
+          <t>Resolved from prior unloaded entry. Was VP/CIO Honda North America since 2022 (cold since Aug 2022). Now SVP Enterprise Transformation &amp; Deputy Lead Global IT - American Honda Motor Company. 2 months in role / 13 yrs in company. Tasks created.</t>
         </is>
       </c>
     </row>
@@ -3203,50 +3228,54 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+      <c r="A58" s="18" t="inlineStr">
         <is>
           <t>Pouria Dehghani</t>
         </is>
       </c>
-      <c r="B58" s="22" t="inlineStr">
-        <is>
-          <t>Unknown - card not loaded</t>
-        </is>
-      </c>
-      <c r="C58" s="22" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D58" s="22" t="inlineStr">
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>Senior Site Reliability Engineer</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Crusoe (kept HubSpot company as Index Exchange per JAM rule)</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>Job Change</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr">
-        <is>
-          <t>NEEDS REVIEW</t>
-        </is>
-      </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
         <is>
           <t>Andy McLean (196669355)</t>
         </is>
       </c>
-      <c r="G58" s="22" t="inlineStr">
-        <is>
-          <t>Sales Nav lazy-load failed</t>
-        </is>
-      </c>
-      <c r="H58" s="23" t="inlineStr">
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>Tasks already created 4/21 (Touch 1 sent + Touch 2 due 5/5). Skipped duplicate creation.</t>
+        </is>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
         <is>
           <t>Pouria Dehghani - HubSpot</t>
         </is>
       </c>
-      <c r="I58" s="22" t="inlineStr"/>
-      <c r="J58" s="22" t="inlineStr">
-        <is>
-          <t>Page 3 result. Was Senior Site Reliability Engineer (Ceph) at Index Exchange. New role/company not loaded. Andy-owned in HubSpot. Manual review needed.</t>
+      <c r="I58" s="18" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J58" s="18" t="inlineStr">
+        <is>
+          <t>Resolved from prior unloaded entry. Senior SRE at Crusoe (AI compute / Bitcoin mining DC). Crusoe is owned by another rep (Brian Charrette). Per JAM rule, kept Andy-owned Index Exchange record. Existing LinkedIn task in flight. Title updated.</t>
         </is>
       </c>
     </row>
@@ -3455,6 +3484,486 @@
       <c r="J63" s="24" t="inlineStr">
         <is>
           <t>Casting producer. Not relevant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="26" t="inlineStr">
+        <is>
+          <t>Darren Wilson</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>Network Security Administrator II</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>Jordan's Furniture</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F64" s="26" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G64" s="26" t="inlineStr">
+        <is>
+          <t>2 tasks created: 4/27 (Touch 1) + 5/11 (Touch 2)</t>
+        </is>
+      </c>
+      <c r="H64" s="27" t="inlineStr">
+        <is>
+          <t>Darren Wilson - HubSpot</t>
+        </is>
+      </c>
+      <c r="I64" s="26" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J64" s="26" t="inlineStr">
+        <is>
+          <t>Promoted internally at Jordan's Furniture from Network Administrator to Network Security Admin II. 2 months in role / 3 yrs in company. Andy already owns. Last contacted 2023-09. Cold reactivation via promotion angle. Title updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>Daryl W Ward</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>Technical Operations Manager</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>IREN (HubSpot kept as Charter Communications)</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F65" s="26" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355) at Charter; IREN owned by Hunter Humphries (204059654)</t>
+        </is>
+      </c>
+      <c r="G65" s="26" t="inlineStr">
+        <is>
+          <t>2 tasks created: 4/27 (Touch 1) + 5/11 (Touch 2)</t>
+        </is>
+      </c>
+      <c r="H65" s="27" t="inlineStr">
+        <is>
+          <t>Daryl Ward - HubSpot</t>
+        </is>
+      </c>
+      <c r="I65" s="26" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J65" s="26" t="inlineStr">
+        <is>
+          <t>Was Director IT at Charter Communications (Andy-owned). Now Technical Operations Mgr at IREN (AI compute/Bitcoin mining DC, Hunter Humphries owns). Per JAM rule, kept HubSpot company as Charter and still created tasks. Strong DIMM history Aug 2024. Title updated. Note: Charter email flagged invalid by ZeroBounce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="28" t="inlineStr">
+        <is>
+          <t>Anthony Steller</t>
+        </is>
+      </c>
+      <c r="B66" s="28" t="inlineStr">
+        <is>
+          <t>Director of Interconnection Strategy + Advisory Board (USNUA)</t>
+        </is>
+      </c>
+      <c r="C66" s="28" t="inlineStr">
+        <is>
+          <t>H5 Data Centers + US Networking User Association</t>
+        </is>
+      </c>
+      <c r="D66" s="28" t="inlineStr">
+        <is>
+          <t>New Role (concurrent advisory)</t>
+        </is>
+      </c>
+      <c r="E66" s="28" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F66" s="28" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355) at H5 Data Centers</t>
+        </is>
+      </c>
+      <c r="G66" s="28" t="inlineStr">
+        <is>
+          <t>No new tasks - already in active engagement (last contacted 2026-03-03)</t>
+        </is>
+      </c>
+      <c r="H66" s="29" t="inlineStr">
+        <is>
+          <t>Anthony Steller - HubSpot</t>
+        </is>
+      </c>
+      <c r="I66" s="28" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J66" s="28" t="inlineStr">
+        <is>
+          <t>Concurrent role: Director Interconnection Strategy at H5 Data Centers (primary, Andy-owned, recently contacted) AND new Advisory Board Member at US Networking User Association (board/volunteer). Already in active outreach - skipped tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="30" t="inlineStr">
+        <is>
+          <t>Steve Drimones</t>
+        </is>
+      </c>
+      <c r="B67" s="30" t="inlineStr">
+        <is>
+          <t>Lead Endpoint Security Engineering</t>
+        </is>
+      </c>
+      <c r="C67" s="30" t="inlineStr">
+        <is>
+          <t>KPMG US (HubSpot at Vornado Realty Trust)</t>
+        </is>
+      </c>
+      <c r="D67" s="30" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E67" s="30" t="inlineStr">
+        <is>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F67" s="30" t="inlineStr">
+        <is>
+          <t>Jason Crisenberry (241105427) - INACTIVE</t>
+        </is>
+      </c>
+      <c r="G67" s="30" t="inlineStr">
+        <is>
+          <t>No tasks - HubSpot record under another rep at prior company</t>
+        </is>
+      </c>
+      <c r="H67" s="31" t="inlineStr">
+        <is>
+          <t>Steve Drimones - HubSpot</t>
+        </is>
+      </c>
+      <c r="I67" s="30" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J67" s="30" t="inlineStr">
+        <is>
+          <t>Was Security Engineer at Vornado Realty Trust under Jason Crisenberry (now inactive owner). Now at KPMG US. Endpoint security is borderline ICP. Owner is inactive so could be reassigned later but not actioning now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>Ted Vaughan</t>
+        </is>
+      </c>
+      <c r="B68" s="30" t="inlineStr">
+        <is>
+          <t>Regional Director, Network Building + Consulting</t>
+        </is>
+      </c>
+      <c r="C68" s="30" t="inlineStr">
+        <is>
+          <t>Network Building + Consulting (NBC LLC)</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>Jim Fulkerson (178980940)</t>
+        </is>
+      </c>
+      <c r="G68" s="30" t="inlineStr">
+        <is>
+          <t>No tasks - contact under another rep (Jim Fulkerson)</t>
+        </is>
+      </c>
+      <c r="H68" s="31" t="inlineStr">
+        <is>
+          <t>Ted Vaughan - HubSpot</t>
+        </is>
+      </c>
+      <c r="I68" s="30" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J68" s="30" t="inlineStr">
+        <is>
+          <t>Promoted from Program Manager to Regional Director at NBC LLC. 2 months in new role / 5 yrs 10 months at company. Owned by Jim Fulkerson - per rules, Excel only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="32" t="inlineStr">
+        <is>
+          <t>James Tuttle</t>
+        </is>
+      </c>
+      <c r="B69" s="32" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>SENTICIT (Roseville, CA)</t>
+        </is>
+      </c>
+      <c r="D69" s="32" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E69" s="32" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="F69" s="32" t="inlineStr">
+        <is>
+          <t>No JAM-owned record; 3 separate James Tuttles in HubSpot (PRTC/Archie Gardner, Penguin Random House/May Jareda, SBCH/Darren Nevolo)</t>
+        </is>
+      </c>
+      <c r="G69" s="32" t="inlineStr">
+        <is>
+          <t>No action - cannot match Sales Nav profile to any HubSpot record</t>
+        </is>
+      </c>
+      <c r="H69" s="32" t="n"/>
+      <c r="I69" s="32" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J69" s="32" t="inlineStr">
+        <is>
+          <t>CIO at SENTICIT (Roseville CA), 1 month in role/company. SENTICIT not in HubSpot. 3 different James Tuttles in HubSpot, none geographically matching Roseville CA. Manual review needed to confirm identity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="28" t="inlineStr">
+        <is>
+          <t>Shawn Pirzada</t>
+        </is>
+      </c>
+      <c r="B70" s="28" t="inlineStr">
+        <is>
+          <t>Sr. Lead Network Engineer</t>
+        </is>
+      </c>
+      <c r="C70" s="28" t="inlineStr">
+        <is>
+          <t>CBTS</t>
+        </is>
+      </c>
+      <c r="D70" s="28" t="inlineStr">
+        <is>
+          <t>Title Refresh</t>
+        </is>
+      </c>
+      <c r="E70" s="28" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F70" s="28" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G70" s="28" t="inlineStr">
+        <is>
+          <t>No new tasks - already actively engaged (last contacted 2026-03-17)</t>
+        </is>
+      </c>
+      <c r="H70" s="29" t="inlineStr">
+        <is>
+          <t>Shawn Pirzada - HubSpot</t>
+        </is>
+      </c>
+      <c r="I70" s="28" t="inlineStr">
+        <is>
+          <t>LinkedIn Profile</t>
+        </is>
+      </c>
+      <c r="J70" s="28" t="inlineStr">
+        <is>
+          <t>Already at CBTS as Sr. Lead Network Engineer. Sales Nav shows 1 month in role/company suggests internal date refresh, not a real change. Andy already owns and recently contacted. No action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="33" t="inlineStr">
+        <is>
+          <t>Kate LoSchiavo</t>
+        </is>
+      </c>
+      <c r="B71" s="33" t="inlineStr">
+        <is>
+          <t>Event Specialist</t>
+        </is>
+      </c>
+      <c r="C71" s="33" t="inlineStr">
+        <is>
+          <t>McDermott Will &amp; Schulte</t>
+        </is>
+      </c>
+      <c r="D71" s="33" t="inlineStr">
+        <is>
+          <t>New Role</t>
+        </is>
+      </c>
+      <c r="E71" s="33" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F71" s="33" t="n"/>
+      <c r="G71" s="33" t="inlineStr">
+        <is>
+          <t>Silent skip - event specialist at law firm, not networking buyer</t>
+        </is>
+      </c>
+      <c r="H71" s="33" t="n"/>
+      <c r="I71" s="33" t="n"/>
+      <c r="J71" s="33" t="inlineStr">
+        <is>
+          <t>Event specialist role. Not relevant to OSI products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="33" t="inlineStr">
+        <is>
+          <t>Katharine Rudzitis</t>
+        </is>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>VP, Direct Originations</t>
+        </is>
+      </c>
+      <c r="C72" s="33" t="inlineStr">
+        <is>
+          <t>Empire Asset Finance, LLC</t>
+        </is>
+      </c>
+      <c r="D72" s="33" t="inlineStr">
+        <is>
+          <t>New Role</t>
+        </is>
+      </c>
+      <c r="E72" s="33" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F72" s="33" t="n"/>
+      <c r="G72" s="33" t="inlineStr">
+        <is>
+          <t>Silent skip - finance/lending role, not networking</t>
+        </is>
+      </c>
+      <c r="H72" s="33" t="n"/>
+      <c r="I72" s="33" t="n"/>
+      <c r="J72" s="33" t="inlineStr">
+        <is>
+          <t>Finance origination role. Not an IT/networking buyer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="33" t="inlineStr">
+        <is>
+          <t>Sara Guerra</t>
+        </is>
+      </c>
+      <c r="B73" s="33" t="inlineStr">
+        <is>
+          <t>Lead Purchasing Supervisor</t>
+        </is>
+      </c>
+      <c r="C73" s="33" t="inlineStr">
+        <is>
+          <t>Thomson Instrument Company</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="inlineStr">
+        <is>
+          <t>New Role</t>
+        </is>
+      </c>
+      <c r="E73" s="33" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F73" s="33" t="n"/>
+      <c r="G73" s="33" t="inlineStr">
+        <is>
+          <t>Silent skip - lab/instrument company procurement, not IT/network</t>
+        </is>
+      </c>
+      <c r="H73" s="33" t="n"/>
+      <c r="I73" s="33" t="n"/>
+      <c r="J73" s="33" t="inlineStr">
+        <is>
+          <t>Procurement at lab instrument firm, not IT/network procurement. Skip.</t>
         </is>
       </c>
     </row>
@@ -3479,14 +3988,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reschedule 142 email-1s from May 19; update 135 HubSpot LinkedIn tasks
</commit_message>
<xml_diff>
--- a/job-change-tracker.xlsx
+++ b/job-change-tracker.xlsx
@@ -156,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -227,6 +227,9 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -592,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3964,6 +3967,266 @@
       <c r="J73" s="33" t="inlineStr">
         <is>
           <t>Procurement at lab instrument firm, not IT/network procurement. Skip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="34" t="inlineStr">
+        <is>
+          <t>Jacob Akcora</t>
+        </is>
+      </c>
+      <c r="B74" s="34" t="inlineStr">
+        <is>
+          <t>Senior Manager of Technology</t>
+        </is>
+      </c>
+      <c r="C74" s="34" t="inlineStr">
+        <is>
+          <t>CSC</t>
+        </is>
+      </c>
+      <c r="D74" s="34" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E74" s="34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F74" s="34" t="inlineStr">
+        <is>
+          <t>Hunter Humphries (204059654)</t>
+        </is>
+      </c>
+      <c r="G74" s="34" t="inlineStr">
+        <is>
+          <t>No tasks - HubSpot record under Hunter Humphries</t>
+        </is>
+      </c>
+      <c r="H74" s="34" t="inlineStr">
+        <is>
+          <t>https://app.hubspot.com/contacts/21878985/record/0-1/464742</t>
+        </is>
+      </c>
+      <c r="I74" s="34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/sales/lead/ACwAAANyKd0BMAe078eFLBtZlenDMVT8Y2lt0hI,NAME_SEARCH,SwUB</t>
+        </is>
+      </c>
+      <c r="J74" s="34" t="inlineStr">
+        <is>
+          <t>Owns Network + HCI platforms at CSC. Record stale (title=Director of IT, email=powerschool.com). Hunter Humphries owns. Excel only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="35" t="inlineStr">
+        <is>
+          <t>Nick Marra</t>
+        </is>
+      </c>
+      <c r="B75" s="35" t="inlineStr">
+        <is>
+          <t>Executive Director - Infrastructure Engineering Senior Manager</t>
+        </is>
+      </c>
+      <c r="C75" s="35" t="inlineStr">
+        <is>
+          <t>Wells Fargo</t>
+        </is>
+      </c>
+      <c r="D75" s="35" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="E75" s="35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F75" s="35" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G75" s="35" t="inlineStr">
+        <is>
+          <t>2 tasks created: 5/11 (Touch 1) + 5/25 (Touch 2). Contact created in HubSpot (ID 220899615264).</t>
+        </is>
+      </c>
+      <c r="H75" s="35" t="inlineStr">
+        <is>
+          <t>https://app.hubspot.com/contacts/21878985/record/0-1/220899615264</t>
+        </is>
+      </c>
+      <c r="I75" s="35" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/sales/lead/ACwAACWmhNgBlqJ8JApqyydWSAyoDU5PoGAYdIA,NAME_SEARCH,9BdI</t>
+        </is>
+      </c>
+      <c r="J75" s="35" t="inlineStr">
+        <is>
+          <t>Promoted to Executive Director Infrastructure Engineering at Wells Fargo Apr 2026. Wells Fargo owned by Andy. Andy messaged March 2026 before promotion. No work email - only nmarra@stevens.edu on file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="36" t="inlineStr">
+        <is>
+          <t>Joseph Abolghasemi</t>
+        </is>
+      </c>
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>Director of Systems Engineering - US</t>
+        </is>
+      </c>
+      <c r="C76" s="36" t="inlineStr">
+        <is>
+          <t>Options Technology</t>
+        </is>
+      </c>
+      <c r="D76" s="36" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E76" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F76" s="36" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G76" s="36" t="inlineStr">
+        <is>
+          <t>No new tasks - 2 active LinkedIn tasks already in flight (due 5/18 + 6/3). Updated company to Options Technology (created in HubSpot ID 54890586191). Updated title.</t>
+        </is>
+      </c>
+      <c r="H76" s="36" t="inlineStr">
+        <is>
+          <t>https://app.hubspot.com/contacts/21878985/record/0-1/43554175763</t>
+        </is>
+      </c>
+      <c r="I76" s="36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/sales/lead/ACwAABGjj90BgDUt2TV60kP0ONdZe_x1U8ENdSc,NAME_SEARCH,9BdI</t>
+        </is>
+      </c>
+      <c r="J76" s="36" t="inlineStr">
+        <is>
+          <t>Was Senior SE at Cravath (3.5 yrs). Returned to Options Technology as Director, Systems Engineering. Active LinkedIn tasks on HubSpot. Company and title updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="36" t="inlineStr">
+        <is>
+          <t>Manikanta Sai Krishna Chillimunta</t>
+        </is>
+      </c>
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>Principal Network Engineer</t>
+        </is>
+      </c>
+      <c r="C77" s="36" t="inlineStr">
+        <is>
+          <t>Autodesk</t>
+        </is>
+      </c>
+      <c r="D77" s="36" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="E77" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F77" s="36" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G77" s="36" t="inlineStr">
+        <is>
+          <t>No new tasks - 2 active LinkedIn tasks already in flight (due 5/15 + 7/31). Already being worked.</t>
+        </is>
+      </c>
+      <c r="H77" s="36" t="inlineStr">
+        <is>
+          <t>https://app.hubspot.com/contacts/21878985/record/0-1/215350258999</t>
+        </is>
+      </c>
+      <c r="I77" s="36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/sales/lead/ACwAABQaI2kBckLpUkGt-DJ_0kbFe5hI3t3SLkY,NAME_SEARCH,9BdI</t>
+        </is>
+      </c>
+      <c r="J77" s="36" t="inlineStr">
+        <is>
+          <t>Promoted from Senior to Principal Network Engineer at Autodesk. CCNP-certified. Active LinkedIn tasks already in HubSpot. Last Sales Nav message 4/30/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="36" t="inlineStr">
+        <is>
+          <t>Antonio Flores</t>
+        </is>
+      </c>
+      <c r="B78" s="36" t="inlineStr">
+        <is>
+          <t>Infrastructure Engineer</t>
+        </is>
+      </c>
+      <c r="C78" s="36" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="D78" s="36" t="inlineStr">
+        <is>
+          <t>Job Change</t>
+        </is>
+      </c>
+      <c r="E78" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F78" s="36" t="inlineStr">
+        <is>
+          <t>Andy McLean (196669355)</t>
+        </is>
+      </c>
+      <c r="G78" s="36" t="inlineStr">
+        <is>
+          <t>No new tasks - 2 active LinkedIn tasks already in flight (due 7/14 + 7/28). Already being worked.</t>
+        </is>
+      </c>
+      <c r="H78" s="36" t="inlineStr">
+        <is>
+          <t>https://app.hubspot.com/contacts/21878985/record/0-1/2685601</t>
+        </is>
+      </c>
+      <c r="I78" s="36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/sales/lead/ACwAABrxIskBcevqM0YToQuHvfeS9aMCVvvo_zE,NAME_SEARCH,9BdI</t>
+        </is>
+      </c>
+      <c r="J78" s="36" t="inlineStr">
+        <is>
+          <t>New role at Datum (data center company) Apr 2026. Prior engagement Oct 2023 (replied). Andy messaged 4/13 and 4/30 before this weekly run. Active LinkedIn tasks on HubSpot.</t>
         </is>
       </c>
     </row>

</xml_diff>